<commit_message>
feat: adding options to save changes
</commit_message>
<xml_diff>
--- a/produtos_new.xlsx
+++ b/produtos_new.xlsx
@@ -413,20 +413,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:C3"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arroz</t>
+          <t>Switch</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22</v>
+        <v>434.52</v>
       </c>
     </row>
     <row r="3">
@@ -435,11 +452,700 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nivea </t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C3" t="n">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>668.84</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Impressora</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2292.03</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Webcam</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3786.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1148.65</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Placa de Vídeo</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3942.76</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Headset</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2091.16</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4021.82</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2239.62</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Carregador</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3855.66</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
         <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cabo HDMI</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2469.86</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>343.9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Carregador</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1581.63</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3958.48</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>531.59</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Pendrive</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4181.72</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roteador</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>4539.53</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Cabo HDMI</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3363.97</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>4726.82</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Smartphone</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3365.32</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Carregador</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>4792.38</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Microfone</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2539.88</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>3774.29</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Placa de Vídeo</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>4542.98</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3598.19</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Cadeira</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1363.08</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Smartphone</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>4050.8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Pendrive</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1711.81</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>350.06</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3305.85</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Impressora</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>978.09</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Mesa</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>164.01</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Gabinete</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>3353.18</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Caixa de Som</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3990.37</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>506.45</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Carregador</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3105</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Cabo HDMI</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2269.97</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>HD Externo</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>227.32</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Scanner</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>4121.16</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Switch</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>279.8</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1184.84</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Mesa</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2745.54</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Carregador</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>3449.51</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1810.61</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HD Externo</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>4885.6</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Smartphone</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>595.16</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Scanner</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>868.63</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Scanner</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2141</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>1767.41</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Placa de Vídeo</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2012.16</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Smartphone</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>3670.75</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Impressora</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>4286.02</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>3560.96</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SSD</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>509.41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>